<commit_message>
docs: finalise project objectives; begin design section
</commit_message>
<xml_diff>
--- a/Questionnaire_Data.xlsx
+++ b/Questionnaire_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Desktop\evac-planner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CAC8CCB-05E4-4254-A7CE-6B62FC8DA2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48732482-7CCF-4C85-BEA2-2D815B9D72F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8985" yWindow="0" windowWidth="11640" windowHeight="13065" firstSheet="2" activeTab="2" xr2:uid="{A878FE0B-7225-47D4-B16F-FD65C796803A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20760" windowHeight="13200" firstSheet="1" activeTab="3" xr2:uid="{A878FE0B-7225-47D4-B16F-FD65C796803A}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -333,9 +333,6 @@
     <t>Q10_TooComplex</t>
   </si>
   <si>
-    <t>Q10_SlowOrFiddly</t>
-  </si>
-  <si>
     <t>Q11_AlgorithmComparison</t>
   </si>
   <si>
@@ -349,6 +346,9 @@
   </si>
   <si>
     <t>Sum</t>
+  </si>
+  <si>
+    <t>Q10_SlowOrTricky</t>
   </si>
 </sst>
 </file>
@@ -723,37 +723,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -1397,6 +1366,7 @@
         <c:crossAx val="1372769072"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="1"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -3565,6 +3535,7 @@
         <c:crossAx val="1368453712"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="1"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -11476,19 +11447,19 @@
         <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -11783,7 +11754,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B12">
         <f>SUM(B$2:B$11)</f>

</xml_diff>